<commit_message>
Air-Way first: unbuildable Air-Way cells take Brennan's value (user Q1)
6405-24-16-O L31 1.75, 6504-24-24 D1 1.312, 6565-10-10 nut hexes 1.000 from the
Brennan TFA catalog (= the values built now), rows marked DimSource BRENNAN;
6405-24-16-O D3 follows the rule (Air-Way 1.14). Regenerated: 236
configurations in 26 roots (+6565, property text only), 0 lost, checks clean,
UNTRACED 0. Dry-run groups rebuilt for 26 roots.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q7fghVUQufSmsb3wBGXToz
</commit_message>
<xml_diff>
--- a/tools/_out/airway_first_20261020/regen/stage/straight/DesignTable_6405_SW2.xlsx
+++ b/tools/_out/airway_first_20261020/regen/stage/straight/DesignTable_6405_SW2.xlsx
@@ -5352,7 +5352,7 @@
         <v>1.75</v>
       </c>
       <c r="W41" t="n">
-        <v>1.08</v>
+        <v>1.14</v>
       </c>
       <c r="X41" t="n">
         <v>0.61</v>
@@ -5389,12 +5389,12 @@
       </c>
       <c r="AE41" t="inlineStr">
         <is>
-          <t>ORB end: sourced; female NPTF: tap drill (AW) + P1 (MS51503 transfer, ASSUMED); L31/hex: Air-Way single source; L31@DRIVE: OMi WebsitePartsInfo2026.xlsx Items!L1802 Overall Length = 1.750 (table had 1); D3@BORE: OMi WebsitePartsInfo2026.xlsx Items!S1802 Side 1 ID = 1.080 (table had 1.14) [user 2026-09-25: OMi dims &gt; Air-Way, ASSUMED] | MODEL: ORB end as 6401; female drill depth = FPT_P1 from the review table (MS51503 P1 max), thread cut to full drill depth (ASSUMPTION); Brennan 5405-08-08 STEP (2026-09-23) confirms 1/2 NPTF port drill depth 0.900 = MS51503 P1 max (VERIFIED for -08 only; thread taper depth in that STEP is 0.750, tap drill dia 0.718, drill point 120 deg); bore D3 from the ORB tip to the pocket bottom</t>
+          <t>[BRENNAN-CELL 2026-10-20: L31@DRIVE] ORB end: sourced; female NPTF: tap drill (AW) + P1 (MS51503 transfer, ASSUMED); L31/hex: Air-Way single source; L31@DRIVE: OMi WebsitePartsInfo2026.xlsx Items!L1802 Overall Length = 1.750 (table had 1); D3@BORE: OMi WebsitePartsInfo2026.xlsx Items!S1802 Side 1 ID = 1.080 (table had 1.14) [user 2026-09-25: OMi dims &gt; Air-Way, ASSUMED]; D3@BORE: Air-Way 1.14 (log (no Air-Way raw extract in the repo); OMi file / Brennan 1.08) [OMi 2026-10-20 (Triveni): Air-Way over Brennan where Air-Way gives a value, incl. the numbers of OMi's website parts file (= Brennan data)]; L31@DRIVE: Brennan TFA catalog p16 table TFA-p016-t01 "MORB-FP STRAIGHT" row 6405-24-16-O col "L LGTH" = 1.75 [user 2026-10-20 Q1: Air-Way value cannot be built -&gt; Brennan] | MODEL: ORB end as 6401; female drill depth = FPT_P1 from the review table (MS51503 P1 max), thread cut to full drill depth (ASSUMPTION); Brennan 5405-08-08 STEP (2026-09-23) confirms 1/2 NPTF port drill depth 0.900 = MS51503 P1 max (VERIFIED for -08 only; thread taper depth in that STEP is 0.750, tap drill dia 0.718, drill point 120 deg); bore D3 from the ORB tip to the pocket bottom</t>
         </is>
       </c>
       <c r="AF41" t="inlineStr">
         <is>
-          <t>D=1.14 equals tap drill and differs from dash-expected bore 1.312 - column bleed suspected, as-printed | AS-PRINTED WARNING: port drill depth P1 1.14 leaves only 0.610 to the far tip, inside the other end's thread/groove region (0.594) - Air-Way L 1.75 looks suspect for this size (built as printed)</t>
+          <t>D=1.14 equals tap drill and differs from dash-expected bore 1.312 - column bleed suspected, as-printed | 2026-10-20 Air-Way first: D3@BORE OMi/Brennan 1.08 -&gt; Air-Way 1.14 | 2026-10-20 L31@DRIVE = Brennan 1.75 (Air-Way 1.0 cannot be built: Air-Way L 1.00 &lt; the 1-NPTF pocket depth 1.14: no room for a bore (generator BLOCKED)) | AS-PRINTED WARNING: port drill depth P1 1.14 leaves only 0.610 to the far tip, inside the other end's thread/groove region (0.594) - Air-Way L 1.75 looks suspect for this size (built as printed)</t>
         </is>
       </c>
       <c r="AG41" t="inlineStr">

</xml_diff>